<commit_message>
Added Django setup module
</commit_message>
<xml_diff>
--- a/Database Example.xlsx
+++ b/Database Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\DEV\HiiT\Python Class 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A4FFCE2-5377-46DE-89C7-9ECF8F1CACD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C2F808-0D12-4262-A2E4-8DC4FBE4EFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B2A0A23B-4769-4EBF-B9BB-9E51834FBC1F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{B2A0A23B-4769-4EBF-B9BB-9E51834FBC1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>ID</t>
   </si>
@@ -51,19 +51,28 @@
     <t>Last name</t>
   </si>
   <si>
-    <t>Order Item</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>userID</t>
+    <t>jge/300</t>
+  </si>
+  <si>
+    <t>Seyi</t>
+  </si>
+  <si>
+    <t>Tinbs</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Stole meat</t>
+  </si>
+  <si>
+    <t>commiter_id</t>
   </si>
 </sst>
 </file>
@@ -435,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{185512F0-610A-496B-AF13-9263B84C1571}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.6328125" customWidth="1"/>
@@ -455,6 +464,20 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -462,30 +485,49 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FADF8E0B-0753-4EED-BFCD-55E2796C5EC1}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
       <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>